<commit_message>
QA pass on iBankNet_CA_Deposits_v1 (0 critical/major) + make guide/corrections links clickable
https://claude.ai/code/session_014WdfNSevF6i6PT6GydKC2F
</commit_message>
<xml_diff>
--- a/research/ibanknet/deliverables/iBankNet_CA_Deposits_v1.xlsx
+++ b/research/ibanknet/deliverables/iBankNet_CA_Deposits_v1.xlsx
@@ -1966,7 +1966,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>—</t>
@@ -1992,7 +1991,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -2220,7 +2218,6 @@
           <t>Phone/branch (no online app for business card)</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -2998,7 +2995,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>NO</t>
@@ -3458,7 +3454,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>—</t>
@@ -3484,7 +3479,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -3828,7 +3822,6 @@
           <t>In-person ('Contact your local branch')</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -4258,7 +4251,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>—</t>
@@ -4284,7 +4276,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -4482,7 +4473,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>—</t>
@@ -4508,7 +4498,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -5286,7 +5275,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>—</t>
@@ -5312,7 +5300,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -5626,7 +5613,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>—</t>
@@ -5648,7 +5634,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -6078,7 +6063,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>—</t>
@@ -6104,7 +6088,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -6418,7 +6401,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>—</t>
@@ -6444,7 +6426,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -6642,7 +6623,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>—</t>
@@ -6668,7 +6648,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -6982,7 +6961,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>—</t>
@@ -7004,7 +6982,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
       <c r="P55" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -7434,7 +7411,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>—</t>
@@ -7456,7 +7432,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
       <c r="P59" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -8234,7 +8209,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>—</t>
@@ -8260,7 +8234,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
       <c r="P66" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -8458,7 +8431,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>—</t>
@@ -8480,7 +8452,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
       <c r="P68" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -9142,7 +9113,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>—</t>
@@ -9164,7 +9134,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
       <c r="P74" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -9246,7 +9215,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>—</t>
@@ -9272,7 +9240,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
       <c r="P75" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -10166,7 +10133,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>NO</t>
@@ -10192,7 +10158,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
       <c r="P83" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -10390,7 +10355,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
           <t>—</t>
@@ -10416,7 +10380,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
       <c r="P85" s="2" t="inlineStr">
         <is>
           <t>Free FICO score on consumer card statements (not Experian as prior noted)</t>
@@ -10992,7 +10955,6 @@
           <t>In-person (banking center / local banker; no online app shown)</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
       <c r="P90" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -11074,7 +11036,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
           <t>—</t>
@@ -11100,7 +11061,6 @@
           <t>Private banker only</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -11530,7 +11490,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
           <t>—</t>
@@ -11556,7 +11515,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr"/>
       <c r="P95" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -11754,7 +11712,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
           <t>NO</t>
@@ -11780,7 +11737,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
       <c r="P97" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -11862,7 +11818,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
           <t>—</t>
@@ -11888,7 +11843,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr"/>
       <c r="P98" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -13478,7 +13432,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
           <t>—</t>
@@ -13500,7 +13453,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O112" t="inlineStr"/>
       <c r="P112" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -13582,7 +13534,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>—</t>
@@ -13604,7 +13555,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O113" t="inlineStr"/>
       <c r="P113" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -13832,7 +13782,6 @@
           <t>Call/Branch</t>
         </is>
       </c>
-      <c r="O115" t="inlineStr"/>
       <c r="P115" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -13914,7 +13863,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>—</t>
@@ -13940,7 +13888,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O116" t="inlineStr"/>
       <c r="P116" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -14138,7 +14085,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>—</t>
@@ -14160,7 +14106,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O118" t="inlineStr"/>
       <c r="P118" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -14242,7 +14187,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>NO</t>
@@ -14268,7 +14212,6 @@
           <t>No (HomeStreet); successor Mechanics Bank: Online via Elan</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr"/>
       <c r="P119" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -14350,7 +14293,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
           <t>—</t>
@@ -14376,7 +14318,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr"/>
       <c r="P120" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -14922,7 +14863,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
           <t>—</t>
@@ -14944,7 +14884,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O125" t="inlineStr"/>
       <c r="P125" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -15258,7 +15197,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr">
         <is>
           <t>—</t>
@@ -15280,7 +15218,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr"/>
       <c r="P128" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -15478,7 +15415,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
           <t>—</t>
@@ -15504,7 +15440,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O130" t="inlineStr"/>
       <c r="P130" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -15586,7 +15521,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr">
         <is>
           <t>—</t>
@@ -15608,7 +15542,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O131" t="inlineStr"/>
       <c r="P131" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -15690,7 +15623,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr">
         <is>
           <t>—</t>
@@ -15716,7 +15648,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O132" t="inlineStr"/>
       <c r="P132" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -15914,7 +15845,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
           <t>—</t>
@@ -15936,7 +15866,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O134" t="inlineStr"/>
       <c r="P134" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -16134,7 +16063,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr">
         <is>
           <t>—</t>
@@ -16156,7 +16084,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O136" t="inlineStr"/>
       <c r="P136" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -16238,7 +16165,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
           <t>—</t>
@@ -16264,7 +16190,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O137" t="inlineStr"/>
       <c r="P137" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -16694,7 +16619,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
           <t>—</t>
@@ -16716,7 +16640,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O141" t="inlineStr"/>
       <c r="P141" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17262,7 +17185,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr">
         <is>
           <t>NO</t>
@@ -17288,7 +17210,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O146" t="inlineStr"/>
       <c r="P146" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17370,7 +17291,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr">
         <is>
           <t>—</t>
@@ -17392,7 +17312,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O147" t="inlineStr"/>
       <c r="P147" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17474,7 +17393,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
       <c r="J148" t="inlineStr">
         <is>
           <t>—</t>
@@ -17500,7 +17418,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O148" t="inlineStr"/>
       <c r="P148" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17582,7 +17499,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
           <t>—</t>
@@ -17608,7 +17524,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O149" t="inlineStr"/>
       <c r="P149" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17806,7 +17721,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr">
         <is>
           <t>—</t>
@@ -17828,7 +17742,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O151" t="inlineStr"/>
       <c r="P151" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -17910,7 +17823,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr">
         <is>
           <t>—</t>
@@ -17932,7 +17844,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O152" t="inlineStr"/>
       <c r="P152" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -18478,7 +18389,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr"/>
       <c r="J157" t="inlineStr">
         <is>
           <t>—</t>
@@ -18504,7 +18414,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O157" t="inlineStr"/>
       <c r="P157" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -18702,7 +18611,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr">
         <is>
           <t>—</t>
@@ -18728,7 +18636,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O159" t="inlineStr"/>
       <c r="P159" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -18810,7 +18717,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr">
         <is>
           <t>NO</t>
@@ -18836,7 +18742,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O160" t="inlineStr"/>
       <c r="P160" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -19034,7 +18939,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr">
         <is>
           <t>—</t>
@@ -19060,7 +18964,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O162" t="inlineStr"/>
       <c r="P162" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -19142,7 +19045,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr"/>
       <c r="J163" t="inlineStr">
         <is>
           <t>—</t>
@@ -19164,7 +19066,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O163" t="inlineStr"/>
       <c r="P163" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -19478,7 +19379,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
           <t>—</t>
@@ -19500,7 +19400,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O166" t="inlineStr"/>
       <c r="P166" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -19582,7 +19481,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I167" t="inlineStr"/>
       <c r="J167" t="inlineStr">
         <is>
           <t>—</t>
@@ -19608,7 +19506,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O167" t="inlineStr"/>
       <c r="P167" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -19690,7 +19587,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
       <c r="J168" t="inlineStr">
         <is>
           <t>—</t>
@@ -19716,7 +19612,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O168" t="inlineStr"/>
       <c r="P168" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -20030,7 +19925,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr"/>
       <c r="J171" t="inlineStr">
         <is>
           <t>—</t>
@@ -20052,7 +19946,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O171" t="inlineStr"/>
       <c r="P171" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -20134,7 +20027,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr">
         <is>
           <t>—</t>
@@ -20156,7 +20048,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O172" t="inlineStr"/>
       <c r="P172" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -20354,7 +20245,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr">
         <is>
           <t>—</t>
@@ -20380,7 +20270,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O174" t="inlineStr"/>
       <c r="P174" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -20810,7 +20699,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>—</t>
@@ -20832,7 +20720,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O178" t="inlineStr"/>
       <c r="P178" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -21146,7 +21033,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr">
         <is>
           <t>not stated</t>
@@ -21258,7 +21144,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr">
         <is>
           <t>—</t>
@@ -21280,7 +21165,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O182" t="inlineStr"/>
       <c r="P182" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -21710,7 +21594,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr">
         <is>
           <t>—</t>
@@ -21736,7 +21619,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O186" t="inlineStr"/>
       <c r="P186" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -21934,7 +21816,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
           <t>—</t>
@@ -21956,7 +21837,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O188" t="inlineStr"/>
       <c r="P188" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -22386,7 +22266,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I192" t="inlineStr"/>
       <c r="J192" t="inlineStr">
         <is>
           <t>—</t>
@@ -22408,7 +22287,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O192" t="inlineStr"/>
       <c r="P192" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -22490,7 +22368,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I193" t="inlineStr"/>
       <c r="J193" t="inlineStr">
         <is>
           <t>—</t>
@@ -22512,7 +22389,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O193" t="inlineStr"/>
       <c r="P193" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -22594,7 +22470,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr">
         <is>
           <t>—</t>
@@ -22616,7 +22491,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O194" t="inlineStr"/>
       <c r="P194" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -22698,7 +22572,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I195" t="inlineStr"/>
       <c r="J195" t="inlineStr">
         <is>
           <t>—</t>
@@ -22724,7 +22597,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O195" t="inlineStr"/>
       <c r="P195" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -22836,7 +22708,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O196" t="inlineStr"/>
       <c r="P196" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -23150,7 +23021,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I199" t="inlineStr"/>
       <c r="J199" t="inlineStr">
         <is>
           <t>—</t>
@@ -23176,7 +23046,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O199" t="inlineStr"/>
       <c r="P199" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -23520,7 +23389,6 @@
           <t>In-person/phone (no online card application)</t>
         </is>
       </c>
-      <c r="O202" t="inlineStr"/>
       <c r="P202" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -23718,7 +23586,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I204" t="inlineStr"/>
       <c r="J204" t="inlineStr">
         <is>
           <t>—</t>
@@ -23744,7 +23611,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O204" t="inlineStr"/>
       <c r="P204" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -23942,7 +23808,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I206" t="inlineStr"/>
       <c r="J206" t="inlineStr">
         <is>
           <t>—</t>
@@ -23968,7 +23833,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O206" t="inlineStr"/>
       <c r="P206" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -24050,7 +23914,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I207" t="inlineStr"/>
       <c r="J207" t="inlineStr">
         <is>
           <t>—</t>
@@ -24072,7 +23935,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O207" t="inlineStr"/>
       <c r="P207" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -24270,7 +24132,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I209" t="inlineStr"/>
       <c r="J209" t="inlineStr">
         <is>
           <t>—</t>
@@ -24296,7 +24157,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O209" t="inlineStr"/>
       <c r="P209" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -24494,7 +24354,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I211" t="inlineStr"/>
       <c r="J211" t="inlineStr">
         <is>
           <t>—</t>
@@ -24516,7 +24375,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O211" t="inlineStr"/>
       <c r="P211" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -24598,7 +24456,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I212" t="inlineStr"/>
       <c r="J212" t="inlineStr">
         <is>
           <t>NO</t>
@@ -24624,7 +24481,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O212" t="inlineStr"/>
       <c r="P212" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -24706,7 +24562,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I213" t="inlineStr"/>
       <c r="J213" t="inlineStr">
         <is>
           <t>—</t>
@@ -24732,7 +24587,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O213" t="inlineStr"/>
       <c r="P213" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -24814,7 +24668,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I214" t="inlineStr"/>
       <c r="J214" t="inlineStr">
         <is>
           <t>—</t>
@@ -24840,7 +24693,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O214" t="inlineStr"/>
       <c r="P214" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -25038,7 +24890,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I216" t="inlineStr"/>
       <c r="J216" t="inlineStr">
         <is>
           <t>—</t>
@@ -25060,7 +24911,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O216" t="inlineStr"/>
       <c r="P216" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -25142,7 +24992,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I217" t="inlineStr"/>
       <c r="J217" t="inlineStr">
         <is>
           <t>—</t>
@@ -25164,7 +25013,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O217" t="inlineStr"/>
       <c r="P217" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -25246,7 +25094,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I218" t="inlineStr"/>
       <c r="J218" t="inlineStr">
         <is>
           <t>—</t>
@@ -25272,7 +25119,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O218" t="inlineStr"/>
       <c r="P218" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -25586,7 +25432,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I221" t="inlineStr"/>
       <c r="J221" t="inlineStr">
         <is>
           <t>—</t>
@@ -25608,7 +25453,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O221" t="inlineStr"/>
       <c r="P221" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -25922,7 +25766,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I224" t="inlineStr"/>
       <c r="J224" t="inlineStr">
         <is>
           <t>—</t>
@@ -25948,7 +25791,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O224" t="inlineStr"/>
       <c r="P224" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26030,7 +25872,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I225" t="inlineStr"/>
       <c r="J225" t="inlineStr">
         <is>
           <t>—</t>
@@ -26052,7 +25893,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O225" t="inlineStr"/>
       <c r="P225" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26134,7 +25974,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I226" t="inlineStr"/>
       <c r="J226" t="inlineStr">
         <is>
           <t>—</t>
@@ -26160,7 +25999,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O226" t="inlineStr"/>
       <c r="P226" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26358,7 +26196,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I228" t="inlineStr"/>
       <c r="J228" t="inlineStr">
         <is>
           <t>—</t>
@@ -26380,7 +26217,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O228" t="inlineStr"/>
       <c r="P228" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26462,7 +26298,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I229" t="inlineStr"/>
       <c r="J229" t="inlineStr">
         <is>
           <t>—</t>
@@ -26488,7 +26323,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O229" t="inlineStr"/>
       <c r="P229" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26802,7 +26636,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I232" t="inlineStr"/>
       <c r="J232" t="inlineStr">
         <is>
           <t>—</t>
@@ -26824,7 +26657,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O232" t="inlineStr"/>
       <c r="P232" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -26906,7 +26738,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I233" t="inlineStr"/>
       <c r="J233" t="inlineStr">
         <is>
           <t>—</t>
@@ -26928,7 +26759,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O233" t="inlineStr"/>
       <c r="P233" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27010,7 +26840,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I234" t="inlineStr"/>
       <c r="J234" t="inlineStr">
         <is>
           <t>—</t>
@@ -27036,7 +26865,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O234" t="inlineStr"/>
       <c r="P234" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -27118,7 +26946,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I235" t="inlineStr"/>
       <c r="J235" t="inlineStr">
         <is>
           <t>—</t>
@@ -27140,7 +26967,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O235" t="inlineStr"/>
       <c r="P235" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27222,7 +27048,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I236" t="inlineStr"/>
       <c r="J236" t="inlineStr">
         <is>
           <t>—</t>
@@ -27248,7 +27073,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O236" t="inlineStr"/>
       <c r="P236" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27330,7 +27154,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I237" t="inlineStr"/>
       <c r="J237" t="inlineStr">
         <is>
           <t>—</t>
@@ -27442,7 +27265,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I238" t="inlineStr"/>
       <c r="J238" t="inlineStr">
         <is>
           <t>—</t>
@@ -27468,7 +27290,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O238" t="inlineStr"/>
       <c r="P238" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27550,7 +27371,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I239" t="inlineStr"/>
       <c r="J239" t="inlineStr">
         <is>
           <t>—</t>
@@ -27572,7 +27392,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O239" t="inlineStr"/>
       <c r="P239" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27654,7 +27473,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I240" t="inlineStr"/>
       <c r="J240" t="inlineStr">
         <is>
           <t>—</t>
@@ -27676,7 +27494,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O240" t="inlineStr"/>
       <c r="P240" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27758,7 +27575,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I241" t="inlineStr"/>
       <c r="J241" t="inlineStr">
         <is>
           <t>—</t>
@@ -27780,7 +27596,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O241" t="inlineStr"/>
       <c r="P241" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27862,7 +27677,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I242" t="inlineStr"/>
       <c r="J242" t="inlineStr">
         <is>
           <t>NO</t>
@@ -27888,7 +27702,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O242" t="inlineStr"/>
       <c r="P242" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -27970,7 +27783,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I243" t="inlineStr"/>
       <c r="J243" t="inlineStr">
         <is>
           <t>—</t>
@@ -27992,7 +27804,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O243" t="inlineStr"/>
       <c r="P243" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -28190,7 +28001,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I245" t="inlineStr"/>
       <c r="J245" t="inlineStr">
         <is>
           <t>—</t>
@@ -28212,7 +28022,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O245" t="inlineStr"/>
       <c r="P245" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -28294,7 +28103,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I246" t="inlineStr"/>
       <c r="J246" t="inlineStr">
         <is>
           <t>—</t>
@@ -28320,7 +28128,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O246" t="inlineStr"/>
       <c r="P246" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -28402,7 +28209,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I247" t="inlineStr"/>
       <c r="J247" t="inlineStr">
         <is>
           <t>—</t>
@@ -28424,7 +28230,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O247" t="inlineStr"/>
       <c r="P247" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -28854,7 +28659,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I251" t="inlineStr"/>
       <c r="J251" t="inlineStr">
         <is>
           <t>—</t>
@@ -28880,7 +28684,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O251" t="inlineStr"/>
       <c r="P251" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -28962,7 +28765,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I252" t="inlineStr"/>
       <c r="J252" t="inlineStr">
         <is>
           <t>—</t>
@@ -28988,7 +28790,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O252" t="inlineStr"/>
       <c r="P252" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29070,7 +28871,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I253" t="inlineStr"/>
       <c r="J253" t="inlineStr">
         <is>
           <t>—</t>
@@ -29092,7 +28892,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O253" t="inlineStr"/>
       <c r="P253" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29174,7 +28973,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I254" t="inlineStr"/>
       <c r="J254" t="inlineStr">
         <is>
           <t>NO</t>
@@ -29200,7 +28998,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O254" t="inlineStr"/>
       <c r="P254" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29282,7 +29079,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I255" t="inlineStr"/>
       <c r="J255" t="inlineStr">
         <is>
           <t>—</t>
@@ -29304,7 +29100,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O255" t="inlineStr"/>
       <c r="P255" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29386,7 +29181,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I256" t="inlineStr"/>
       <c r="J256" t="inlineStr">
         <is>
           <t>—</t>
@@ -29408,7 +29202,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O256" t="inlineStr"/>
       <c r="P256" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29490,7 +29283,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I257" t="inlineStr"/>
       <c r="J257" t="inlineStr">
         <is>
           <t>—</t>
@@ -29512,7 +29304,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O257" t="inlineStr"/>
       <c r="P257" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -29594,7 +29385,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I258" t="inlineStr"/>
       <c r="J258" t="inlineStr">
         <is>
           <t>—</t>
@@ -29616,7 +29406,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O258" t="inlineStr"/>
       <c r="P258" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -30046,7 +29835,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I262" t="inlineStr"/>
       <c r="J262" t="inlineStr">
         <is>
           <t>—</t>
@@ -30072,7 +29860,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O262" t="inlineStr"/>
       <c r="P262" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -30154,7 +29941,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I263" t="inlineStr"/>
       <c r="J263" t="inlineStr">
         <is>
           <t>—</t>
@@ -30176,7 +29962,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O263" t="inlineStr"/>
       <c r="P263" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -30258,7 +30043,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I264" t="inlineStr"/>
       <c r="J264" t="inlineStr">
         <is>
           <t>—</t>
@@ -30284,7 +30068,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O264" t="inlineStr"/>
       <c r="P264" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -30482,7 +30265,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I266" t="inlineStr"/>
       <c r="J266" t="inlineStr">
         <is>
           <t>—</t>
@@ -30508,7 +30290,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O266" t="inlineStr"/>
       <c r="P266" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -30590,7 +30371,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I267" t="inlineStr"/>
       <c r="J267" t="inlineStr">
         <is>
           <t>—</t>
@@ -30616,7 +30396,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O267" t="inlineStr"/>
       <c r="P267" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -30814,7 +30593,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I269" t="inlineStr"/>
       <c r="J269" t="inlineStr">
         <is>
           <t>—</t>
@@ -30836,7 +30614,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O269" t="inlineStr"/>
       <c r="P269" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -30918,7 +30695,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I270" t="inlineStr"/>
       <c r="J270" t="inlineStr">
         <is>
           <t>—</t>
@@ -30940,7 +30716,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O270" t="inlineStr"/>
       <c r="P270" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31022,7 +30797,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I271" t="inlineStr"/>
       <c r="J271" t="inlineStr">
         <is>
           <t>—</t>
@@ -31044,7 +30818,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O271" t="inlineStr"/>
       <c r="P271" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31126,7 +30899,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I272" t="inlineStr"/>
       <c r="J272" t="inlineStr">
         <is>
           <t>—</t>
@@ -31148,7 +30920,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O272" t="inlineStr"/>
       <c r="P272" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31230,7 +31001,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I273" t="inlineStr"/>
       <c r="J273" t="inlineStr">
         <is>
           <t>NO</t>
@@ -31256,7 +31026,6 @@
           <t>No (business); consumer card via branch/phone 626-965-6230</t>
         </is>
       </c>
-      <c r="O273" t="inlineStr"/>
       <c r="P273" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31338,7 +31107,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I274" t="inlineStr"/>
       <c r="J274" t="inlineStr">
         <is>
           <t>—</t>
@@ -31364,7 +31132,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O274" t="inlineStr"/>
       <c r="P274" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31476,7 +31243,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O275" t="inlineStr"/>
       <c r="P275" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31558,7 +31324,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I276" t="inlineStr"/>
       <c r="J276" t="inlineStr">
         <is>
           <t>—</t>
@@ -31580,7 +31345,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O276" t="inlineStr"/>
       <c r="P276" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31662,7 +31426,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I277" t="inlineStr"/>
       <c r="J277" t="inlineStr">
         <is>
           <t>—</t>
@@ -31684,7 +31447,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O277" t="inlineStr"/>
       <c r="P277" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31766,7 +31528,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr">
         <is>
           <t>—</t>
@@ -31788,7 +31549,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O278" t="inlineStr"/>
       <c r="P278" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31870,7 +31630,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I279" t="inlineStr"/>
       <c r="J279" t="inlineStr">
         <is>
           <t>—</t>
@@ -31892,7 +31651,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O279" t="inlineStr"/>
       <c r="P279" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -31974,7 +31732,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I280" t="inlineStr"/>
       <c r="J280" t="inlineStr">
         <is>
           <t>—</t>
@@ -31996,7 +31753,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O280" t="inlineStr"/>
       <c r="P280" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32078,7 +31834,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I281" t="inlineStr"/>
       <c r="J281" t="inlineStr">
         <is>
           <t>—</t>
@@ -32104,7 +31859,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O281" t="inlineStr"/>
       <c r="P281" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32186,7 +31940,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I282" t="inlineStr"/>
       <c r="J282" t="inlineStr">
         <is>
           <t>—</t>
@@ -32208,7 +31961,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O282" t="inlineStr"/>
       <c r="P282" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32290,7 +32042,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I283" t="inlineStr"/>
       <c r="J283" t="inlineStr">
         <is>
           <t>—</t>
@@ -32316,7 +32067,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O283" t="inlineStr"/>
       <c r="P283" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32514,7 +32264,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr"/>
       <c r="J285" t="inlineStr">
         <is>
           <t>—</t>
@@ -32536,7 +32285,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O285" t="inlineStr"/>
       <c r="P285" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32618,7 +32366,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I286" t="inlineStr"/>
       <c r="J286" t="inlineStr">
         <is>
           <t>—</t>
@@ -32640,7 +32387,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O286" t="inlineStr"/>
       <c r="P286" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32722,7 +32468,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I287" t="inlineStr"/>
       <c r="J287" t="inlineStr">
         <is>
           <t>—</t>
@@ -32744,7 +32489,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O287" t="inlineStr"/>
       <c r="P287" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -32826,7 +32570,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I288" t="inlineStr"/>
       <c r="J288" t="inlineStr">
         <is>
           <t>—</t>
@@ -32848,7 +32591,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O288" t="inlineStr"/>
       <c r="P288" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -33046,7 +32788,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I290" t="inlineStr"/>
       <c r="J290" t="inlineStr">
         <is>
           <t>—</t>
@@ -33072,7 +32813,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O290" t="inlineStr"/>
       <c r="P290" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -33154,7 +32894,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
       <c r="J291" t="inlineStr">
         <is>
           <t>—</t>
@@ -33176,7 +32915,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O291" t="inlineStr"/>
       <c r="P291" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -33606,7 +33344,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I295" t="inlineStr"/>
       <c r="J295" t="inlineStr">
         <is>
           <t>—</t>
@@ -33628,7 +33365,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O295" t="inlineStr"/>
       <c r="P295" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -33826,7 +33562,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I297" t="inlineStr"/>
       <c r="J297" t="inlineStr">
         <is>
           <t>—</t>
@@ -33848,7 +33583,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O297" t="inlineStr"/>
       <c r="P297" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -33930,7 +33664,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I298" t="inlineStr"/>
       <c r="J298" t="inlineStr">
         <is>
           <t>—</t>
@@ -33952,7 +33685,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O298" t="inlineStr"/>
       <c r="P298" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34034,7 +33766,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I299" t="inlineStr"/>
       <c r="J299" t="inlineStr">
         <is>
           <t>—</t>
@@ -34060,7 +33791,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O299" t="inlineStr"/>
       <c r="P299" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34142,7 +33872,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I300" t="inlineStr"/>
       <c r="J300" t="inlineStr">
         <is>
           <t>—</t>
@@ -34254,7 +33983,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I301" t="inlineStr"/>
       <c r="J301" t="inlineStr">
         <is>
           <t>—</t>
@@ -34276,7 +34004,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O301" t="inlineStr"/>
       <c r="P301" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34358,7 +34085,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I302" t="inlineStr"/>
       <c r="J302" t="inlineStr">
         <is>
           <t>—</t>
@@ -34380,7 +34106,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O302" t="inlineStr"/>
       <c r="P302" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34462,7 +34187,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I303" t="inlineStr"/>
       <c r="J303" t="inlineStr">
         <is>
           <t>—</t>
@@ -34484,7 +34208,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O303" t="inlineStr"/>
       <c r="P303" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34566,7 +34289,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I304" t="inlineStr"/>
       <c r="J304" t="inlineStr">
         <is>
           <t>—</t>
@@ -34592,7 +34314,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O304" t="inlineStr"/>
       <c r="P304" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34674,7 +34395,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I305" t="inlineStr"/>
       <c r="J305" t="inlineStr">
         <is>
           <t>—</t>
@@ -34696,7 +34416,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O305" t="inlineStr"/>
       <c r="P305" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34778,7 +34497,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I306" t="inlineStr"/>
       <c r="J306" t="inlineStr">
         <is>
           <t>—</t>
@@ -34800,7 +34518,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O306" t="inlineStr"/>
       <c r="P306" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34882,7 +34599,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I307" t="inlineStr"/>
       <c r="J307" t="inlineStr">
         <is>
           <t>—</t>
@@ -34904,7 +34620,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O307" t="inlineStr"/>
       <c r="P307" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -34986,7 +34701,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I308" t="inlineStr"/>
       <c r="J308" t="inlineStr">
         <is>
           <t>—</t>
@@ -35008,7 +34722,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O308" t="inlineStr"/>
       <c r="P308" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35090,7 +34803,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I309" t="inlineStr"/>
       <c r="J309" t="inlineStr">
         <is>
           <t>—</t>
@@ -35112,7 +34824,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O309" t="inlineStr"/>
       <c r="P309" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35310,7 +35021,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I311" t="inlineStr"/>
       <c r="J311" t="inlineStr">
         <is>
           <t>—</t>
@@ -35332,7 +35042,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O311" t="inlineStr"/>
       <c r="P311" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35414,7 +35123,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I312" t="inlineStr"/>
       <c r="J312" t="inlineStr">
         <is>
           <t>—</t>
@@ -35440,7 +35148,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O312" t="inlineStr"/>
       <c r="P312" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -35522,7 +35229,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I313" t="inlineStr"/>
       <c r="J313" t="inlineStr">
         <is>
           <t>—</t>
@@ -35548,7 +35254,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O313" t="inlineStr"/>
       <c r="P313" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35630,7 +35335,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I314" t="inlineStr"/>
       <c r="J314" t="inlineStr">
         <is>
           <t>—</t>
@@ -35652,7 +35356,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O314" t="inlineStr"/>
       <c r="P314" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35734,7 +35437,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I315" t="inlineStr"/>
       <c r="J315" t="inlineStr">
         <is>
           <t>—</t>
@@ -35756,7 +35458,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O315" t="inlineStr"/>
       <c r="P315" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35838,7 +35539,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I316" t="inlineStr"/>
       <c r="J316" t="inlineStr">
         <is>
           <t>—</t>
@@ -35860,7 +35560,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O316" t="inlineStr"/>
       <c r="P316" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -35942,7 +35641,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I317" t="inlineStr"/>
       <c r="J317" t="inlineStr">
         <is>
           <t>—</t>
@@ -35968,7 +35666,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O317" t="inlineStr"/>
       <c r="P317" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36050,7 +35747,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I318" t="inlineStr"/>
       <c r="J318" t="inlineStr">
         <is>
           <t>—</t>
@@ -36072,7 +35768,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O318" t="inlineStr"/>
       <c r="P318" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36154,7 +35849,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I319" t="inlineStr"/>
       <c r="J319" t="inlineStr">
         <is>
           <t>—</t>
@@ -36176,7 +35870,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O319" t="inlineStr"/>
       <c r="P319" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36258,7 +35951,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I320" t="inlineStr"/>
       <c r="J320" t="inlineStr">
         <is>
           <t>—</t>
@@ -36284,7 +35976,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O320" t="inlineStr"/>
       <c r="P320" s="2" t="inlineStr">
         <is>
           <t>Prior mentor 'Experian' DP remains uncorroborated</t>
@@ -36366,7 +36057,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I321" t="inlineStr"/>
       <c r="J321" t="inlineStr">
         <is>
           <t>—</t>
@@ -36392,7 +36082,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O321" t="inlineStr"/>
       <c r="P321" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36590,7 +36279,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I323" t="inlineStr"/>
       <c r="J323" t="inlineStr">
         <is>
           <t>—</t>
@@ -36612,7 +36300,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O323" t="inlineStr"/>
       <c r="P323" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36694,7 +36381,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I324" t="inlineStr"/>
       <c r="J324" t="inlineStr">
         <is>
           <t>—</t>
@@ -36716,7 +36402,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O324" t="inlineStr"/>
       <c r="P324" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36798,7 +36483,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I325" t="inlineStr"/>
       <c r="J325" t="inlineStr">
         <is>
           <t>—</t>
@@ -36820,7 +36504,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O325" t="inlineStr"/>
       <c r="P325" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -36902,7 +36585,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I326" t="inlineStr"/>
       <c r="J326" t="inlineStr">
         <is>
           <t>—</t>
@@ -36924,7 +36606,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O326" t="inlineStr"/>
       <c r="P326" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37006,7 +36687,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr"/>
       <c r="J327" t="inlineStr">
         <is>
           <t>—</t>
@@ -37028,7 +36708,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O327" t="inlineStr"/>
       <c r="P327" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37110,7 +36789,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I328" t="inlineStr"/>
       <c r="J328" t="inlineStr">
         <is>
           <t>—</t>
@@ -37136,7 +36814,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O328" t="inlineStr"/>
       <c r="P328" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37218,7 +36895,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I329" t="inlineStr"/>
       <c r="J329" t="inlineStr">
         <is>
           <t>—</t>
@@ -37240,7 +36916,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O329" t="inlineStr"/>
       <c r="P329" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37438,7 +37113,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I331" t="inlineStr"/>
       <c r="J331" t="inlineStr">
         <is>
           <t>—</t>
@@ -37460,7 +37134,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O331" t="inlineStr"/>
       <c r="P331" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37542,7 +37215,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I332" t="inlineStr"/>
       <c r="J332" t="inlineStr">
         <is>
           <t>—</t>
@@ -37564,7 +37236,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O332" t="inlineStr"/>
       <c r="P332" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37646,7 +37317,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I333" t="inlineStr"/>
       <c r="J333" t="inlineStr">
         <is>
           <t>—</t>
@@ -37672,7 +37342,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O333" t="inlineStr"/>
       <c r="P333" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37754,7 +37423,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I334" t="inlineStr"/>
       <c r="J334" t="inlineStr">
         <is>
           <t>—</t>
@@ -37776,7 +37444,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O334" t="inlineStr"/>
       <c r="P334" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37858,7 +37525,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I335" t="inlineStr"/>
       <c r="J335" t="inlineStr">
         <is>
           <t>—</t>
@@ -37880,7 +37546,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O335" t="inlineStr"/>
       <c r="P335" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -37962,7 +37627,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I336" t="inlineStr"/>
       <c r="J336" t="inlineStr">
         <is>
           <t>—</t>
@@ -37988,7 +37652,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O336" t="inlineStr"/>
       <c r="P336" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38070,7 +37733,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I337" t="inlineStr"/>
       <c r="J337" t="inlineStr">
         <is>
           <t>NO</t>
@@ -38096,7 +37758,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O337" t="inlineStr"/>
       <c r="P337" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38178,7 +37839,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I338" t="inlineStr"/>
       <c r="J338" t="inlineStr">
         <is>
           <t>—</t>
@@ -38200,7 +37860,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O338" t="inlineStr"/>
       <c r="P338" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38282,7 +37941,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I339" t="inlineStr"/>
       <c r="J339" t="inlineStr">
         <is>
           <t>—</t>
@@ -38308,7 +37966,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O339" t="inlineStr"/>
       <c r="P339" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38390,7 +38047,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I340" t="inlineStr"/>
       <c r="J340" t="inlineStr">
         <is>
           <t>—</t>
@@ -38412,7 +38068,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O340" t="inlineStr"/>
       <c r="P340" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38640,7 +38295,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O342" t="inlineStr"/>
       <c r="P342" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38722,7 +38376,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I343" t="inlineStr"/>
       <c r="J343" t="inlineStr">
         <is>
           <t>—</t>
@@ -38744,7 +38397,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O343" t="inlineStr"/>
       <c r="P343" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -38942,7 +38594,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr"/>
       <c r="J345" t="inlineStr">
         <is>
           <t>—</t>
@@ -38968,7 +38619,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O345" t="inlineStr"/>
       <c r="P345" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39050,7 +38700,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I346" t="inlineStr"/>
       <c r="J346" t="inlineStr">
         <is>
           <t>—</t>
@@ -39072,7 +38721,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O346" t="inlineStr"/>
       <c r="P346" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39154,7 +38802,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I347" t="inlineStr"/>
       <c r="J347" t="inlineStr">
         <is>
           <t>—</t>
@@ -39176,7 +38823,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O347" t="inlineStr"/>
       <c r="P347" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39258,7 +38904,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I348" t="inlineStr"/>
       <c r="J348" t="inlineStr">
         <is>
           <t>—</t>
@@ -39284,7 +38929,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O348" t="inlineStr"/>
       <c r="P348" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39366,7 +39010,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I349" t="inlineStr"/>
       <c r="J349" t="inlineStr">
         <is>
           <t>—</t>
@@ -39388,7 +39031,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O349" t="inlineStr"/>
       <c r="P349" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39470,7 +39112,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I350" t="inlineStr"/>
       <c r="J350" t="inlineStr">
         <is>
           <t>—</t>
@@ -39492,7 +39133,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O350" t="inlineStr"/>
       <c r="P350" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39574,7 +39214,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr"/>
       <c r="J351" t="inlineStr">
         <is>
           <t>—</t>
@@ -39596,7 +39235,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O351" t="inlineStr"/>
       <c r="P351" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39678,7 +39316,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I352" t="inlineStr"/>
       <c r="J352" t="inlineStr">
         <is>
           <t>—</t>
@@ -39700,7 +39337,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O352" t="inlineStr"/>
       <c r="P352" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39782,7 +39418,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I353" t="inlineStr"/>
       <c r="J353" t="inlineStr">
         <is>
           <t>—</t>
@@ -39808,7 +39443,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O353" t="inlineStr"/>
       <c r="P353" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39890,7 +39524,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I354" t="inlineStr"/>
       <c r="J354" t="inlineStr">
         <is>
           <t>—</t>
@@ -39912,7 +39545,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O354" t="inlineStr"/>
       <c r="P354" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -39994,7 +39626,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I355" t="inlineStr"/>
       <c r="J355" t="inlineStr">
         <is>
           <t>—</t>
@@ -40016,7 +39647,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O355" t="inlineStr"/>
       <c r="P355" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40330,7 +39960,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I358" t="inlineStr"/>
       <c r="J358" t="inlineStr">
         <is>
           <t>—</t>
@@ -40352,7 +39981,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O358" t="inlineStr"/>
       <c r="P358" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40434,7 +40062,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I359" t="inlineStr"/>
       <c r="J359" t="inlineStr">
         <is>
           <t>—</t>
@@ -40456,7 +40083,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O359" t="inlineStr"/>
       <c r="P359" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40538,7 +40164,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr"/>
       <c r="J360" t="inlineStr">
         <is>
           <t>—</t>
@@ -40560,7 +40185,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O360" t="inlineStr"/>
       <c r="P360" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40642,7 +40266,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I361" t="inlineStr"/>
       <c r="J361" t="inlineStr">
         <is>
           <t>—</t>
@@ -40668,7 +40291,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O361" t="inlineStr"/>
       <c r="P361" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -40750,7 +40372,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I362" t="inlineStr"/>
       <c r="J362" t="inlineStr">
         <is>
           <t>—</t>
@@ -40776,7 +40397,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O362" t="inlineStr"/>
       <c r="P362" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40858,7 +40478,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I363" t="inlineStr"/>
       <c r="J363" t="inlineStr">
         <is>
           <t>—</t>
@@ -40880,7 +40499,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O363" t="inlineStr"/>
       <c r="P363" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -40962,7 +40580,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr"/>
       <c r="J364" t="inlineStr">
         <is>
           <t>—</t>
@@ -40984,7 +40601,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O364" t="inlineStr"/>
       <c r="P364" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41066,7 +40682,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I365" t="inlineStr"/>
       <c r="J365" t="inlineStr">
         <is>
           <t>—</t>
@@ -41088,7 +40703,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O365" t="inlineStr"/>
       <c r="P365" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41170,7 +40784,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I366" t="inlineStr"/>
       <c r="J366" t="inlineStr">
         <is>
           <t>—</t>
@@ -41196,7 +40809,6 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="O366" t="inlineStr"/>
       <c r="P366" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
@@ -41278,7 +40890,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I367" t="inlineStr"/>
       <c r="J367" t="inlineStr">
         <is>
           <t>—</t>
@@ -41300,7 +40911,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O367" t="inlineStr"/>
       <c r="P367" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41382,7 +40992,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I368" t="inlineStr"/>
       <c r="J368" t="inlineStr">
         <is>
           <t>—</t>
@@ -41404,7 +41013,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O368" t="inlineStr"/>
       <c r="P368" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41486,7 +41094,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I369" t="inlineStr"/>
       <c r="J369" t="inlineStr">
         <is>
           <t>—</t>
@@ -41508,7 +41115,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O369" t="inlineStr"/>
       <c r="P369" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41590,7 +41196,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I370" t="inlineStr"/>
       <c r="J370" t="inlineStr">
         <is>
           <t>—</t>
@@ -41616,7 +41221,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O370" t="inlineStr"/>
       <c r="P370" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41698,7 +41302,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I371" t="inlineStr"/>
       <c r="J371" t="inlineStr">
         <is>
           <t>—</t>
@@ -41720,7 +41323,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O371" t="inlineStr"/>
       <c r="P371" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41802,7 +41404,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I372" t="inlineStr"/>
       <c r="J372" t="inlineStr">
         <is>
           <t>—</t>
@@ -41824,7 +41425,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O372" t="inlineStr"/>
       <c r="P372" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -41906,7 +41506,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I373" t="inlineStr"/>
       <c r="J373" t="inlineStr">
         <is>
           <t>—</t>
@@ -41928,7 +41527,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O373" t="inlineStr"/>
       <c r="P373" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42126,7 +41724,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I375" t="inlineStr"/>
       <c r="J375" t="inlineStr">
         <is>
           <t>—</t>
@@ -42148,7 +41745,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O375" t="inlineStr"/>
       <c r="P375" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42230,7 +41826,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I376" t="inlineStr"/>
       <c r="J376" t="inlineStr">
         <is>
           <t>—</t>
@@ -42252,7 +41847,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O376" t="inlineStr"/>
       <c r="P376" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42334,7 +41928,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I377" t="inlineStr"/>
       <c r="J377" t="inlineStr">
         <is>
           <t>—</t>
@@ -42360,7 +41953,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O377" t="inlineStr"/>
       <c r="P377" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42442,7 +42034,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I378" t="inlineStr"/>
       <c r="J378" t="inlineStr">
         <is>
           <t>—</t>
@@ -42464,7 +42055,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O378" t="inlineStr"/>
       <c r="P378" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42546,7 +42136,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I379" t="inlineStr"/>
       <c r="J379" t="inlineStr">
         <is>
           <t>—</t>
@@ -42568,7 +42157,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O379" t="inlineStr"/>
       <c r="P379" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42650,7 +42238,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I380" t="inlineStr"/>
       <c r="J380" t="inlineStr">
         <is>
           <t>—</t>
@@ -42672,7 +42259,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O380" t="inlineStr"/>
       <c r="P380" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42754,7 +42340,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I381" t="inlineStr"/>
       <c r="J381" t="inlineStr">
         <is>
           <t>—</t>
@@ -42776,7 +42361,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O381" t="inlineStr"/>
       <c r="P381" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42858,7 +42442,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I382" t="inlineStr"/>
       <c r="J382" t="inlineStr">
         <is>
           <t>—</t>
@@ -42880,7 +42463,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O382" t="inlineStr"/>
       <c r="P382" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -42962,7 +42544,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I383" t="inlineStr"/>
       <c r="J383" t="inlineStr">
         <is>
           <t>—</t>
@@ -42984,7 +42565,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O383" t="inlineStr"/>
       <c r="P383" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43066,7 +42646,6 @@
           <t>UNCLEAR</t>
         </is>
       </c>
-      <c r="I384" t="inlineStr"/>
       <c r="J384" t="inlineStr">
         <is>
           <t>—</t>
@@ -43092,7 +42671,6 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="O384" t="inlineStr"/>
       <c r="P384" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43174,7 +42752,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I385" t="inlineStr"/>
       <c r="J385" t="inlineStr">
         <is>
           <t>—</t>
@@ -43196,7 +42773,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O385" t="inlineStr"/>
       <c r="P385" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43278,7 +42854,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I386" t="inlineStr"/>
       <c r="J386" t="inlineStr">
         <is>
           <t>—</t>
@@ -43300,7 +42875,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O386" t="inlineStr"/>
       <c r="P386" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43382,7 +42956,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I387" t="inlineStr"/>
       <c r="J387" t="inlineStr">
         <is>
           <t>—</t>
@@ -43404,7 +42977,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O387" t="inlineStr"/>
       <c r="P387" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43486,7 +43058,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I388" t="inlineStr"/>
       <c r="J388" t="inlineStr">
         <is>
           <t>—</t>
@@ -43508,7 +43079,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O388" t="inlineStr"/>
       <c r="P388" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43590,7 +43160,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I389" t="inlineStr"/>
       <c r="J389" t="inlineStr">
         <is>
           <t>—</t>
@@ -43612,7 +43181,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O389" t="inlineStr"/>
       <c r="P389" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43694,7 +43262,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I390" t="inlineStr"/>
       <c r="J390" t="inlineStr">
         <is>
           <t>—</t>
@@ -43716,7 +43283,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O390" t="inlineStr"/>
       <c r="P390" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43798,7 +43364,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I391" t="inlineStr"/>
       <c r="J391" t="inlineStr">
         <is>
           <t>—</t>
@@ -43824,7 +43389,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O391" t="inlineStr"/>
       <c r="P391" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -43906,7 +43470,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I392" t="inlineStr"/>
       <c r="J392" t="inlineStr">
         <is>
           <t>—</t>
@@ -43928,7 +43491,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O392" t="inlineStr"/>
       <c r="P392" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44010,7 +43572,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I393" t="inlineStr"/>
       <c r="J393" t="inlineStr">
         <is>
           <t>—</t>
@@ -44032,7 +43593,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O393" t="inlineStr"/>
       <c r="P393" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44114,7 +43674,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I394" t="inlineStr"/>
       <c r="J394" t="inlineStr">
         <is>
           <t>—</t>
@@ -44136,7 +43695,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O394" t="inlineStr"/>
       <c r="P394" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44218,7 +43776,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I395" t="inlineStr"/>
       <c r="J395" t="inlineStr">
         <is>
           <t>—</t>
@@ -44240,7 +43797,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O395" t="inlineStr"/>
       <c r="P395" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44322,7 +43878,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I396" t="inlineStr"/>
       <c r="J396" t="inlineStr">
         <is>
           <t>—</t>
@@ -44344,7 +43899,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O396" t="inlineStr"/>
       <c r="P396" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44426,7 +43980,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I397" t="inlineStr"/>
       <c r="J397" t="inlineStr">
         <is>
           <t>—</t>
@@ -44448,7 +44001,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O397" t="inlineStr"/>
       <c r="P397" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44530,7 +44082,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I398" t="inlineStr"/>
       <c r="J398" t="inlineStr">
         <is>
           <t>—</t>
@@ -44556,7 +44107,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O398" t="inlineStr"/>
       <c r="P398" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44638,7 +44188,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I399" t="inlineStr"/>
       <c r="J399" t="inlineStr">
         <is>
           <t>—</t>
@@ -44660,7 +44209,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O399" t="inlineStr"/>
       <c r="P399" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44742,7 +44290,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I400" t="inlineStr"/>
       <c r="J400" t="inlineStr">
         <is>
           <t>—</t>
@@ -44764,7 +44311,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O400" t="inlineStr"/>
       <c r="P400" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44846,7 +44392,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I401" t="inlineStr"/>
       <c r="J401" t="inlineStr">
         <is>
           <t>—</t>
@@ -44868,7 +44413,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O401" t="inlineStr"/>
       <c r="P401" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -44950,7 +44494,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I402" t="inlineStr"/>
       <c r="J402" t="inlineStr">
         <is>
           <t>—</t>
@@ -44972,7 +44515,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O402" t="inlineStr"/>
       <c r="P402" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45054,7 +44596,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I403" t="inlineStr"/>
       <c r="J403" t="inlineStr">
         <is>
           <t>—</t>
@@ -45076,7 +44617,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O403" t="inlineStr"/>
       <c r="P403" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45158,7 +44698,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I404" t="inlineStr"/>
       <c r="J404" t="inlineStr">
         <is>
           <t>—</t>
@@ -45180,7 +44719,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O404" t="inlineStr"/>
       <c r="P404" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45262,7 +44800,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I405" t="inlineStr"/>
       <c r="J405" t="inlineStr">
         <is>
           <t>—</t>
@@ -45288,7 +44825,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O405" t="inlineStr"/>
       <c r="P405" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45370,7 +44906,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I406" t="inlineStr"/>
       <c r="J406" t="inlineStr">
         <is>
           <t>—</t>
@@ -45392,7 +44927,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O406" t="inlineStr"/>
       <c r="P406" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45474,7 +45008,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I407" t="inlineStr"/>
       <c r="J407" t="inlineStr">
         <is>
           <t>—</t>
@@ -45500,7 +45033,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O407" t="inlineStr"/>
       <c r="P407" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45582,7 +45114,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I408" t="inlineStr"/>
       <c r="J408" t="inlineStr">
         <is>
           <t>—</t>
@@ -45604,7 +45135,6 @@
           <t>Call</t>
         </is>
       </c>
-      <c r="O408" t="inlineStr"/>
       <c r="P408" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45686,7 +45216,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I409" t="inlineStr"/>
       <c r="J409" t="inlineStr">
         <is>
           <t>—</t>
@@ -45708,7 +45237,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O409" t="inlineStr"/>
       <c r="P409" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45790,7 +45318,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I410" t="inlineStr"/>
       <c r="J410" t="inlineStr">
         <is>
           <t>NO</t>
@@ -45816,7 +45343,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="O410" t="inlineStr"/>
       <c r="P410" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -45898,7 +45424,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I411" t="inlineStr"/>
       <c r="J411" t="inlineStr">
         <is>
           <t>—</t>
@@ -45920,7 +45445,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O411" t="inlineStr"/>
       <c r="P411" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46002,7 +45526,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I412" t="inlineStr"/>
       <c r="J412" t="inlineStr">
         <is>
           <t>—</t>
@@ -46024,7 +45547,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O412" t="inlineStr"/>
       <c r="P412" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46106,7 +45628,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I413" t="inlineStr"/>
       <c r="J413" t="inlineStr">
         <is>
           <t>—</t>
@@ -46128,7 +45649,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O413" t="inlineStr"/>
       <c r="P413" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46194,7 +45714,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E414" t="inlineStr"/>
       <c r="F414" s="10" t="n">
         <v>0</v>
       </c>
@@ -46206,7 +45725,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I414" t="inlineStr"/>
       <c r="J414" t="inlineStr">
         <is>
           <t>—</t>
@@ -46232,7 +45750,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O414" t="inlineStr"/>
       <c r="P414" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46298,7 +45815,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E415" t="inlineStr"/>
       <c r="F415" s="10" t="n">
         <v>0</v>
       </c>
@@ -46310,7 +45826,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I415" t="inlineStr"/>
       <c r="J415" t="inlineStr">
         <is>
           <t>—</t>
@@ -46336,7 +45851,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O415" t="inlineStr"/>
       <c r="P415" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46402,7 +45916,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E416" t="inlineStr"/>
       <c r="F416" s="10" t="n">
         <v>0</v>
       </c>
@@ -46414,7 +45927,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I416" t="inlineStr"/>
       <c r="J416" t="inlineStr">
         <is>
           <t>—</t>
@@ -46440,7 +45952,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O416" t="inlineStr"/>
       <c r="P416" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46522,7 +46033,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I417" t="inlineStr"/>
       <c r="J417" t="inlineStr">
         <is>
           <t>—</t>
@@ -46548,7 +46058,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="O417" t="inlineStr"/>
       <c r="P417" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46630,7 +46139,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I418" t="inlineStr"/>
       <c r="J418" t="inlineStr">
         <is>
           <t>—</t>
@@ -46656,7 +46164,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O418" t="inlineStr"/>
       <c r="P418" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -46970,7 +46477,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I421" t="inlineStr"/>
       <c r="J421" t="inlineStr">
         <is>
           <t>—</t>
@@ -46992,7 +46498,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O421" t="inlineStr"/>
       <c r="P421" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47074,7 +46579,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I422" t="inlineStr"/>
       <c r="J422" t="inlineStr">
         <is>
           <t>—</t>
@@ -47096,7 +46600,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O422" t="inlineStr"/>
       <c r="P422" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47178,7 +46681,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I423" t="inlineStr"/>
       <c r="J423" t="inlineStr">
         <is>
           <t>—</t>
@@ -47204,7 +46706,6 @@
           <t>N/M</t>
         </is>
       </c>
-      <c r="O423" t="inlineStr"/>
       <c r="P423" s="2" t="inlineStr">
         <is>
           <t>N/M</t>
@@ -47300,7 +46801,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E425" t="inlineStr"/>
       <c r="F425" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47314,7 +46814,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I425" t="inlineStr"/>
       <c r="J425" t="inlineStr">
         <is>
           <t>—</t>
@@ -47340,7 +46839,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O425" t="inlineStr"/>
       <c r="P425" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47406,7 +46904,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E426" t="inlineStr"/>
       <c r="F426" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47420,7 +46917,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I426" t="inlineStr"/>
       <c r="J426" t="inlineStr">
         <is>
           <t>—</t>
@@ -47446,7 +46942,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O426" t="inlineStr"/>
       <c r="P426" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47512,7 +47007,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E427" t="inlineStr"/>
       <c r="F427" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47526,7 +47020,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I427" t="inlineStr"/>
       <c r="J427" t="inlineStr">
         <is>
           <t>—</t>
@@ -47552,7 +47045,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O427" t="inlineStr"/>
       <c r="P427" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47618,7 +47110,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47632,7 +47123,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I428" t="inlineStr"/>
       <c r="J428" t="inlineStr">
         <is>
           <t>—</t>
@@ -47658,7 +47148,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O428" t="inlineStr"/>
       <c r="P428" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47724,7 +47213,6 @@
           <t>City Of Industry</t>
         </is>
       </c>
-      <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47738,7 +47226,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I429" t="inlineStr"/>
       <c r="J429" t="inlineStr">
         <is>
           <t>—</t>
@@ -47764,7 +47251,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O429" t="inlineStr"/>
       <c r="P429" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47830,7 +47316,6 @@
           <t>Alhambra</t>
         </is>
       </c>
-      <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47844,7 +47329,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I430" t="inlineStr"/>
       <c r="J430" t="inlineStr">
         <is>
           <t>—</t>
@@ -47870,7 +47354,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O430" t="inlineStr"/>
       <c r="P430" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -47936,7 +47419,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -47950,7 +47432,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I431" t="inlineStr"/>
       <c r="J431" t="inlineStr">
         <is>
           <t>—</t>
@@ -47976,7 +47457,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O431" t="inlineStr"/>
       <c r="P431" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48042,7 +47522,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48056,7 +47535,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I432" t="inlineStr"/>
       <c r="J432" t="inlineStr">
         <is>
           <t>—</t>
@@ -48082,7 +47560,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O432" t="inlineStr"/>
       <c r="P432" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48148,7 +47625,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48162,7 +47638,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I433" t="inlineStr"/>
       <c r="J433" t="inlineStr">
         <is>
           <t>—</t>
@@ -48188,7 +47663,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O433" t="inlineStr"/>
       <c r="P433" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48254,7 +47728,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48268,7 +47741,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I434" t="inlineStr"/>
       <c r="J434" t="inlineStr">
         <is>
           <t>—</t>
@@ -48294,7 +47766,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O434" t="inlineStr"/>
       <c r="P434" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48360,7 +47831,6 @@
           <t>Pasadena</t>
         </is>
       </c>
-      <c r="E435" t="inlineStr"/>
       <c r="F435" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48374,7 +47844,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I435" t="inlineStr"/>
       <c r="J435" t="inlineStr">
         <is>
           <t>—</t>
@@ -48400,7 +47869,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O435" t="inlineStr"/>
       <c r="P435" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48466,7 +47934,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48480,7 +47947,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I436" t="inlineStr"/>
       <c r="J436" t="inlineStr">
         <is>
           <t>—</t>
@@ -48506,7 +47972,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O436" t="inlineStr"/>
       <c r="P436" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48572,7 +48037,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48586,7 +48050,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I437" t="inlineStr"/>
       <c r="J437" t="inlineStr">
         <is>
           <t>—</t>
@@ -48612,7 +48075,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O437" t="inlineStr"/>
       <c r="P437" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48678,7 +48140,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48692,7 +48153,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I438" t="inlineStr"/>
       <c r="J438" t="inlineStr">
         <is>
           <t>—</t>
@@ -48718,7 +48178,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O438" t="inlineStr"/>
       <c r="P438" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48784,7 +48243,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E439" t="inlineStr"/>
       <c r="F439" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48798,7 +48256,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I439" t="inlineStr"/>
       <c r="J439" t="inlineStr">
         <is>
           <t>—</t>
@@ -48824,7 +48281,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O439" t="inlineStr"/>
       <c r="P439" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48890,7 +48346,6 @@
           <t>San Jose</t>
         </is>
       </c>
-      <c r="E440" t="inlineStr"/>
       <c r="F440" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -48904,7 +48359,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I440" t="inlineStr"/>
       <c r="J440" t="inlineStr">
         <is>
           <t>—</t>
@@ -48930,7 +48384,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O440" t="inlineStr"/>
       <c r="P440" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -48996,7 +48449,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E441" t="inlineStr"/>
       <c r="F441" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49010,7 +48462,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I441" t="inlineStr"/>
       <c r="J441" t="inlineStr">
         <is>
           <t>—</t>
@@ -49036,7 +48487,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O441" t="inlineStr"/>
       <c r="P441" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49102,7 +48552,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49116,7 +48565,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I442" t="inlineStr"/>
       <c r="J442" t="inlineStr">
         <is>
           <t>—</t>
@@ -49142,7 +48590,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O442" t="inlineStr"/>
       <c r="P442" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49208,7 +48655,6 @@
           <t>Alhambra</t>
         </is>
       </c>
-      <c r="E443" t="inlineStr"/>
       <c r="F443" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49222,7 +48668,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I443" t="inlineStr"/>
       <c r="J443" t="inlineStr">
         <is>
           <t>—</t>
@@ -49248,7 +48693,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O443" t="inlineStr"/>
       <c r="P443" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49314,7 +48758,6 @@
           <t>Alhambra</t>
         </is>
       </c>
-      <c r="E444" t="inlineStr"/>
       <c r="F444" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49328,7 +48771,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I444" t="inlineStr"/>
       <c r="J444" t="inlineStr">
         <is>
           <t>—</t>
@@ -49354,7 +48796,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O444" t="inlineStr"/>
       <c r="P444" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49420,7 +48861,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E445" t="inlineStr"/>
       <c r="F445" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49434,7 +48874,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I445" t="inlineStr"/>
       <c r="J445" t="inlineStr">
         <is>
           <t>—</t>
@@ -49460,7 +48899,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O445" t="inlineStr"/>
       <c r="P445" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49526,7 +48964,6 @@
           <t>Irvine</t>
         </is>
       </c>
-      <c r="E446" t="inlineStr"/>
       <c r="F446" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49540,7 +48977,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I446" t="inlineStr"/>
       <c r="J446" t="inlineStr">
         <is>
           <t>—</t>
@@ -49566,7 +49002,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O446" t="inlineStr"/>
       <c r="P446" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49632,7 +49067,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E447" t="inlineStr"/>
       <c r="F447" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49646,7 +49080,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I447" t="inlineStr"/>
       <c r="J447" t="inlineStr">
         <is>
           <t>—</t>
@@ -49672,7 +49105,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O447" t="inlineStr"/>
       <c r="P447" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49738,7 +49170,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E448" t="inlineStr"/>
       <c r="F448" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49752,7 +49183,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I448" t="inlineStr"/>
       <c r="J448" t="inlineStr">
         <is>
           <t>—</t>
@@ -49778,7 +49208,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O448" t="inlineStr"/>
       <c r="P448" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49844,7 +49273,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E449" t="inlineStr"/>
       <c r="F449" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49858,7 +49286,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I449" t="inlineStr"/>
       <c r="J449" t="inlineStr">
         <is>
           <t>—</t>
@@ -49884,7 +49311,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O449" t="inlineStr"/>
       <c r="P449" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -49950,7 +49376,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E450" t="inlineStr"/>
       <c r="F450" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -49964,7 +49389,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I450" t="inlineStr"/>
       <c r="J450" t="inlineStr">
         <is>
           <t>—</t>
@@ -49990,7 +49414,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O450" t="inlineStr"/>
       <c r="P450" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -50056,7 +49479,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E451" t="inlineStr"/>
       <c r="F451" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -50070,7 +49492,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I451" t="inlineStr"/>
       <c r="J451" t="inlineStr">
         <is>
           <t>—</t>
@@ -50096,7 +49517,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O451" t="inlineStr"/>
       <c r="P451" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -50162,7 +49582,6 @@
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="E452" t="inlineStr"/>
       <c r="F452" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -50176,7 +49595,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I452" t="inlineStr"/>
       <c r="J452" t="inlineStr">
         <is>
           <t>—</t>
@@ -50202,7 +49620,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O452" t="inlineStr"/>
       <c r="P452" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -50268,7 +49685,6 @@
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="E453" t="inlineStr"/>
       <c r="F453" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -50282,7 +49698,6 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I453" t="inlineStr"/>
       <c r="J453" t="inlineStr">
         <is>
           <t>—</t>
@@ -50308,7 +49723,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O453" t="inlineStr"/>
       <c r="P453" s="2" t="inlineStr">
         <is>
           <t>—</t>
@@ -51279,7 +50693,7 @@
           <t>OK - bankofhope.com = Bank of Hope (LA)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>https://www.bankofhope.com/business-banking/credit-cards | https://www.mycardapply.com/synindex/?ecdma-lc=37106&amp;ecid=OTHE_25940&amp;offertype=0#business</t>
         </is>
@@ -51319,7 +50733,7 @@
           <t>OK - fmb.com = F&amp;M Bank Long Beach (main-office Long Beach; investors.fmb.com FMBL). NOT fm.bank / fmbnc.com / fmbanktrust.bank twins</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>https://www.fmb.com/business/business-credit-card | https://creditcardlearnmore.com/11t3/index?ecdma-lc=31463&amp;ecid=OTHE_25940</t>
         </is>
@@ -51359,7 +50773,7 @@
           <t>No twin issue (formerly Manufacturers Bank)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>https://www.smbcmanubank.com/business-and-commercial/borrow/business-lending/business-credit-cards</t>
         </is>
@@ -51399,7 +50813,7 @@
           <t>FAIL in prior (prior site = missionbank.bank = Mission Bank Bakersfield; correct site = missionfed.com San Diego)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>https://www.missionfed.com/business/; https://www.missionbank.bank/business/business-credit-cards; google SERP</t>
         </is>
@@ -51439,7 +50853,7 @@
           <t>OK - kinecta.org genuine Kinecta FCU site</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>https://www.kinecta.org/credit-card/mypro</t>
         </is>
@@ -51479,7 +50893,7 @@
           <t>OK - Elan co-brand portal carries Westamerica branding at lc=12109; westamerica.com 403 bot-block</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>https://creditcardlearnmore.com/11t3/index?ecdma-lc=12109</t>
         </is>
@@ -51519,7 +50933,7 @@
           <t>OK — communitywestbank.com Fresno CA (distinct from Community West CU Michigan + West Bank Iowa twins in search results)</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>https://www.cardaccount.net/application/f87a3255c0/business/new | https://www.communitywestbank.com/business-banking/business-online-banking/business-credit-cards</t>
         </is>
@@ -51559,7 +50973,7 @@
           <t>MISMATCH FIXED - prior row used pbofca.com (Partners Bank of California) for Partners FCU; correct site is partnersfcu.org</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>https://www.partnersfcu.org/</t>
         </is>
@@ -51599,7 +51013,7 @@
           <t>OK - coastccu.org = Coast Central CU Eureka</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>https://www.coastccu.org/business/business-credit-cards/ | https://www.coastccu.org/business/</t>
         </is>
@@ -51639,7 +51053,7 @@
           <t>TWIN FIXED — amerfirst.org (Brea CA CU) vs afnb.com (American First National Bank TX) vs americafirst.com (America First CU, Utah)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>https://www.amerfirst.org/products/business-services; https://www.amerfirst.org/</t>
         </is>
@@ -51679,7 +51093,7 @@
           <t>OK - redwoodcapitalbank.com = Redwood Capital Bank Eureka</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>https://www.redwoodcapitalbank.com/business/business-credit-cards</t>
         </is>
@@ -51719,7 +51133,7 @@
           <t>OK — sunflowerbank.com (also operates as First National 1870)</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="13" t="inlineStr">
         <is>
           <t>https://www.sunflowerbank.com/business/business-accounts/credit-cards; https://www.sunflowerbank.com/Ungrouped-Content/Terms-Conditions/Credit-Card-Terms-Conditions/Corporate-Visa-Credit-Card</t>
         </is>
@@ -51759,7 +51173,7 @@
           <t>OK — legacybankca.com (Murrieta CA); prior already excluded out-of-state Legacy Bank twins (CO/WI)</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>https://www.legacybankca.com/; https://www.legacybankca.com/loans/commercial-lending</t>
         </is>
@@ -51799,7 +51213,7 @@
           <t>FAILED in prior / corrected: GVFCU Manteca = goldenvalleyfcu.org; goldenvalley.bank = Golden Valley Bank Chico (separate FDIC bank)</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>https://goldenvalleyfcu.org/ | https://www.yelp.com/biz/golden-valley-federal-credit-union-manteca</t>
         </is>
@@ -51839,7 +51253,7 @@
           <t>CHANGED — domain redirects to metrocitybank.bank (Doraville GA)</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>https://www.metrocitybank.bank/; https://www.sec.gov/Archives/edgar/data/0001747068/000110465926057876/mcbs-20260331x10q.htm</t>
         </is>
@@ -51852,6 +51266,23 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H16"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>